<commit_message>
allure report and config file added
</commit_message>
<xml_diff>
--- a/TestData/excel.xlsx
+++ b/TestData/excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sriram-HP\Documents\Playwright_ts\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8632B085-0E37-456D-A10D-1993AAE349FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19C25F25-EA43-4926-857D-4B500CFC252D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="20">
   <si>
     <t>password</t>
   </si>
@@ -40,9 +40,6 @@
   </si>
   <si>
     <t>Rock_1986</t>
-  </si>
-  <si>
-    <t>ZARA COAT 3</t>
   </si>
   <si>
     <t>cvv</t>
@@ -426,22 +423,22 @@
         <v>1</v>
       </c>
       <c r="D1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
+        <v>16</v>
+      </c>
+      <c r="I1" t="s">
         <v>7</v>
-      </c>
-      <c r="H1" t="s">
-        <v>17</v>
-      </c>
-      <c r="I1" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
@@ -452,10 +449,10 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E2" s="1">
         <v>14</v>
@@ -464,13 +461,13 @@
         <v>123</v>
       </c>
       <c r="G2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I2" t="s">
         <v>9</v>
-      </c>
-      <c r="H2" t="s">
-        <v>18</v>
-      </c>
-      <c r="I2" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
@@ -481,10 +478,10 @@
         <v>4</v>
       </c>
       <c r="C3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E3" s="1">
         <v>16</v>
@@ -493,13 +490,13 @@
         <v>345</v>
       </c>
       <c r="G3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H3" t="s">
+        <v>18</v>
+      </c>
+      <c r="I3" t="s">
         <v>19</v>
-      </c>
-      <c r="I3" t="s">
-        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>